<commit_message>
chore: archivos de datos y versiones supabase actualizados
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/seguimiento_operacional.xlsx
+++ b/public/seguimiento_operacional.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fchnew-my.sharepoint.com/personal/emilio_lopez_fch_cl/Documents/Documentos/Proyectos/gestion-proyectos-fch/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="8_{44A8C3A5-2FD1-450C-A58C-EBAB01C8E818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0635B682-16C9-4E55-B278-12D1F83FF1C9}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="8_{44A8C3A5-2FD1-450C-A58C-EBAB01C8E818}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2CCA7CAD-2FE0-4D89-96E8-65A065B59458}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DDE99ACA-4FAD-4A17-96E2-0DF5B1B5DD9D}"/>
   </bookViews>
@@ -87,7 +87,17 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="42" formatCode="_ &quot;$&quot;* #,##0_ ;_ &quot;$&quot;* \-#,##0_ ;_ &quot;$&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -113,13 +123,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moneda [0]" xfId="1" builtinId="7"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -492,168 +505,170 @@
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="1">
         <v>6000000</v>
       </c>
-      <c r="C2">
-        <v>22084910</v>
-      </c>
-      <c r="D2">
-        <v>1214545</v>
-      </c>
-      <c r="E2">
-        <v>-17299455</v>
-      </c>
-      <c r="F2">
-        <v>31000000</v>
-      </c>
-      <c r="G2">
-        <v>27520182</v>
-      </c>
-      <c r="H2">
-        <v>5000000</v>
-      </c>
-      <c r="I2">
-        <v>-1520182</v>
+      <c r="C2" s="1">
+        <v>29723051</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1292689</v>
+      </c>
+      <c r="E2" s="1">
+        <v>-25015740</v>
+      </c>
+      <c r="F2" s="1">
+        <v>42000000</v>
+      </c>
+      <c r="G2" s="1">
+        <v>36660487</v>
+      </c>
+      <c r="H2" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="I2" s="1">
+        <v>-4660487</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
-      <c r="C3">
-        <v>53746425</v>
-      </c>
-      <c r="D3">
-        <v>3756333</v>
-      </c>
-      <c r="E3">
-        <v>-57502758</v>
-      </c>
-      <c r="G3">
-        <v>60819486</v>
-      </c>
-      <c r="H3">
-        <v>3430623</v>
-      </c>
-      <c r="I3">
-        <v>-64250109</v>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1">
+        <v>69870960</v>
+      </c>
+      <c r="D3" s="1">
+        <v>4884998</v>
+      </c>
+      <c r="E3" s="1">
+        <v>-74755958</v>
+      </c>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1">
+        <v>79190252</v>
+      </c>
+      <c r="H3" s="1">
+        <v>6097911</v>
+      </c>
+      <c r="I3" s="1">
+        <v>-85288163</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="B4">
-        <v>227563354</v>
-      </c>
-      <c r="C4">
-        <v>80468490</v>
-      </c>
-      <c r="D4">
-        <v>151803724.16000003</v>
-      </c>
-      <c r="E4">
-        <v>-4708860.1600000262</v>
-      </c>
-      <c r="F4">
-        <v>399966902</v>
-      </c>
-      <c r="G4">
-        <v>101340868</v>
-      </c>
-      <c r="H4">
-        <v>296287921</v>
-      </c>
-      <c r="I4">
-        <v>2338113</v>
+      <c r="B4" s="1">
+        <v>340522999</v>
+      </c>
+      <c r="C4" s="1">
+        <v>108891003</v>
+      </c>
+      <c r="D4" s="1">
+        <v>233765691.40000004</v>
+      </c>
+      <c r="E4" s="1">
+        <v>-2133695.4000000358</v>
+      </c>
+      <c r="F4" s="1">
+        <v>583415413</v>
+      </c>
+      <c r="G4" s="1">
+        <v>140592775</v>
+      </c>
+      <c r="H4" s="1">
+        <v>421160348</v>
+      </c>
+      <c r="I4" s="1">
+        <v>21662290</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
-      <c r="B5">
-        <v>58512105</v>
-      </c>
-      <c r="C5">
-        <v>121310190</v>
-      </c>
-      <c r="D5">
-        <v>19389256.079999998</v>
-      </c>
-      <c r="E5">
-        <v>-82187341.079999983</v>
-      </c>
-      <c r="F5">
-        <v>99833333</v>
-      </c>
-      <c r="G5">
-        <v>134204418</v>
-      </c>
-      <c r="H5">
-        <v>6030000</v>
-      </c>
-      <c r="I5">
-        <v>-40401085</v>
+      <c r="B5" s="1">
+        <v>120661255</v>
+      </c>
+      <c r="C5" s="1">
+        <v>162342972</v>
+      </c>
+      <c r="D5" s="1">
+        <v>83309564</v>
+      </c>
+      <c r="E5" s="1">
+        <v>-124991281</v>
+      </c>
+      <c r="F5" s="1">
+        <v>199443333</v>
+      </c>
+      <c r="G5" s="1">
+        <v>181023516</v>
+      </c>
+      <c r="H5" s="1">
+        <v>65839000</v>
+      </c>
+      <c r="I5" s="1">
+        <v>-47419183</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B6">
-        <v>676438075</v>
-      </c>
-      <c r="C6">
-        <v>151214146</v>
-      </c>
-      <c r="D6">
-        <v>522767792.75999987</v>
-      </c>
-      <c r="E6">
-        <v>2456136.2400001287</v>
-      </c>
-      <c r="F6">
-        <v>719195117</v>
-      </c>
-      <c r="G6">
-        <v>155495157</v>
-      </c>
-      <c r="H6">
-        <v>526600000</v>
-      </c>
-      <c r="I6">
-        <v>37099960</v>
+      <c r="B6" s="1">
+        <v>981637498</v>
+      </c>
+      <c r="C6" s="1">
+        <v>196405180</v>
+      </c>
+      <c r="D6" s="1">
+        <v>690165629.01999986</v>
+      </c>
+      <c r="E6" s="1">
+        <v>95066688.980000138</v>
+      </c>
+      <c r="F6" s="1">
+        <v>896823489</v>
+      </c>
+      <c r="G6" s="1">
+        <v>207326876</v>
+      </c>
+      <c r="H6" s="1">
+        <v>640030000</v>
+      </c>
+      <c r="I6" s="1">
+        <v>49466613</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>5</v>
       </c>
-      <c r="B7">
-        <v>98469983</v>
-      </c>
-      <c r="C7">
-        <v>83897973</v>
-      </c>
-      <c r="D7">
-        <v>8175793.3949999996</v>
-      </c>
-      <c r="E7">
-        <v>6396216.6050000042</v>
-      </c>
-      <c r="F7">
-        <v>127191047</v>
-      </c>
-      <c r="G7">
-        <v>86104554</v>
-      </c>
-      <c r="H7">
-        <v>12846219</v>
-      </c>
-      <c r="I7">
-        <v>28240274</v>
+      <c r="B7" s="1">
+        <v>130079437</v>
+      </c>
+      <c r="C7" s="1">
+        <v>114445077</v>
+      </c>
+      <c r="D7" s="1">
+        <v>9172933.8099999987</v>
+      </c>
+      <c r="E7" s="1">
+        <v>6461426.1899999976</v>
+      </c>
+      <c r="F7" s="1">
+        <v>167749770</v>
+      </c>
+      <c r="G7" s="1">
+        <v>114657264</v>
+      </c>
+      <c r="H7" s="1">
+        <v>14475323</v>
+      </c>
+      <c r="I7" s="1">
+        <v>38617183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>